<commit_message>
updated and not live 28 oct
</commit_message>
<xml_diff>
--- a/frontend/public/sku-information-template.xlsx
+++ b/frontend/public/sku-information-template.xlsx
@@ -9,12 +9,12 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="122211"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t xml:space="preserve">S. No. </t>
   </si>
@@ -50,6 +50,9 @@
   </si>
   <si>
     <t>In Transit Units</t>
+  </si>
+  <si>
+    <t>Product Status</t>
   </si>
 </sst>
 </file>
@@ -186,9 +189,9 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -497,15 +500,19 @@
   <dimension ref="A1:M22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.5703125" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" customWidth="1"/>
+    <col min="4" max="4" width="5.28515625" customWidth="1"/>
+    <col min="5" max="5" width="7.85546875" customWidth="1"/>
+    <col min="6" max="6" width="7.7109375" customWidth="1"/>
     <col min="7" max="7" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.140625" customWidth="1"/>
+    <col min="11" max="11" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -536,16 +543,18 @@
       <c r="I1" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="J1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="14" t="s">
+      <c r="K1" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="14" t="s">
+      <c r="L1" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="12"/>
+      <c r="M1" s="14" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="5"/>
@@ -560,6 +569,7 @@
       <c r="J2" s="4"/>
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
+      <c r="M2" s="4"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
@@ -574,6 +584,7 @@
       <c r="J3" s="4"/>
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
+      <c r="M3" s="4"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
@@ -588,6 +599,7 @@
       <c r="J4" s="4"/>
       <c r="K4" s="3"/>
       <c r="L4" s="3"/>
+      <c r="M4" s="4"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
@@ -602,6 +614,7 @@
       <c r="J5" s="4"/>
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
+      <c r="M5" s="4"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
@@ -616,6 +629,7 @@
       <c r="J6" s="4"/>
       <c r="K6" s="3"/>
       <c r="L6" s="3"/>
+      <c r="M6" s="4"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
@@ -630,6 +644,7 @@
       <c r="J7" s="4"/>
       <c r="K7" s="3"/>
       <c r="L7" s="3"/>
+      <c r="M7" s="4"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
@@ -644,6 +659,7 @@
       <c r="J8" s="4"/>
       <c r="K8" s="3"/>
       <c r="L8" s="3"/>
+      <c r="M8" s="4"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="5"/>
@@ -658,6 +674,7 @@
       <c r="J9" s="4"/>
       <c r="K9" s="3"/>
       <c r="L9" s="3"/>
+      <c r="M9" s="4"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
@@ -672,6 +689,7 @@
       <c r="J10" s="4"/>
       <c r="K10" s="3"/>
       <c r="L10" s="3"/>
+      <c r="M10" s="4"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
@@ -686,6 +704,7 @@
       <c r="J11" s="4"/>
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
+      <c r="M11" s="4"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="5"/>
@@ -700,6 +719,7 @@
       <c r="J12" s="4"/>
       <c r="K12" s="3"/>
       <c r="L12" s="3"/>
+      <c r="M12" s="4"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="5"/>
@@ -714,6 +734,7 @@
       <c r="J13" s="4"/>
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
+      <c r="M13" s="4"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>
@@ -728,6 +749,7 @@
       <c r="J14" s="4"/>
       <c r="K14" s="3"/>
       <c r="L14" s="3"/>
+      <c r="M14" s="4"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
@@ -742,6 +764,7 @@
       <c r="J15" s="4"/>
       <c r="K15" s="3"/>
       <c r="L15" s="3"/>
+      <c r="M15" s="4"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="5"/>
@@ -756,8 +779,9 @@
       <c r="J16" s="4"/>
       <c r="K16" s="3"/>
       <c r="L16" s="3"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M16" s="4"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="10"/>
       <c r="B17" s="8"/>
       <c r="C17" s="7"/>
@@ -770,8 +794,9 @@
       <c r="J17" s="4"/>
       <c r="K17" s="3"/>
       <c r="L17" s="3"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M17" s="4"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -784,8 +809,9 @@
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
       <c r="L18" s="1"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M18" s="1"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -798,8 +824,9 @@
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
       <c r="L19" s="1"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M19" s="1"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -812,8 +839,9 @@
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
       <c r="L20" s="1"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M20" s="1"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -826,8 +854,9 @@
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
       <c r="L21" s="1"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M21" s="1"/>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -840,8 +869,14 @@
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
       <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Choose Active or Discontinued." sqref="M2:M17">
+      <formula1>"Active,Discontinued"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>